<commit_message>
Stage 8 fixes: F-011
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/Development/EP11/Compatibility/Bench_Sheets/EP11_compatibility-matrix_092526_interim.xlsx
+++ b/output/archive/DurnesswickData/Development/EP11/Compatibility/Bench_Sheets/EP11_compatibility-matrix_092526_interim.xlsx
@@ -863,12 +863,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Appearance at 2 weeks</t>
+          <t>Appearance at recorded pull</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Status / source</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Colour change. Under investigation</t>
+          <t>Prepared and on stress; observation date in Stress log/source bench sheet. Recipe card under DF26-01022 carries drug/excipient weight proportions and blend-specific start date; elapsed stress time not transcribed.</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>As Blend 1, lower intensity</t>
+          <t>Prepared and on stress; observation date in Stress log/source bench sheet. Recipe card under DF26-01022 carries drug/excipient weight proportions and blend-specific start date; elapsed stress time not transcribed.</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Reference blend</t>
+          <t>Prepared and on stress; observation date in Stress log/source bench sheet. Recipe card under DF26-01022 carries drug/excipient weight proportions and blend-specific start date; elapsed stress time not transcribed.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,11 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>T0 preparation only; awaiting storage slot, not placed on stress. Blend-specific recipe card under DF26-01022 carries weight proportions.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -985,7 +989,11 @@
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting preparation and storage slot; no stress start.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -996,13 +1004,17 @@
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting recipe/preparation and storage slot; no stress start.</t>
+        </is>
+      </c>
     </row>
     <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Stress analyses for Blends 4 to 6 pending.</t>
+          <t>Blends 1–3 on stress; analytical follow-up pending. Blend 4 prepared at T0 only; Blends 5–6 unprepared. No two-week duration inferred without the source start date.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
@@ -1027,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1046,7 +1058,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Observation date</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1170,6 +1182,24 @@
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Recipe / start provenance</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Blend-specific recipe cards under DF26-01022</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Consult weight proportions and actual stress-start entries; elapsed time is not calculated here.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1223,7 +1253,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Alternative filler is in the stress set now. No conclusions until the two-week and four-week pulls are in.</t>
+          <t>Alternative filler remains under evaluation. Blend 4 has a T0 preparation observation only and awaits a storage slot; it has not started stress. Blend 5 awaits preparation and slots; Blend 6 awaits recipe/preparation and slots.</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1265,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Stress samples for Blends 4 to 6 to be prepared once the sample store confirms slots. Final matrix not issued.</t>
+          <t>Blends 1–3 were prepared and placed on stress; start dates and drug/excipient weight proportions remain on blend-specific recipe cards under DF26-01022. Stress log dates are observation dates, not start dates. Prepare/start Blends 4–6 as slots permit; final matrix not issued.</t>
         </is>
       </c>
     </row>

</xml_diff>